<commit_message>
logica para la actualizacio de los xlsx terminada. falta hacerlo para el minorista, y subir al drive
</commit_message>
<xml_diff>
--- a/LISTAS/BISAGRA LIBRO-5005.xlsx
+++ b/LISTAS/BISAGRA LIBRO-5005.xlsx
@@ -761,7 +761,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="10" t="n">
-        <v>45163.60820518138</v>
+        <v>45163.60820518518</v>
       </c>
     </row>
     <row r="2">
@@ -771,10 +771,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="24" t="inlineStr">
         <is>
@@ -817,18 +813,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
@@ -860,7 +844,7 @@
       </c>
       <c r="C26" s="20" t="n"/>
       <c r="D26" s="22" t="n">
-        <v>523.784</v>
+        <v>633.7786400000001</v>
       </c>
       <c r="E26" s="23" t="n"/>
       <c r="F26" s="23" t="n"/>
@@ -879,7 +863,7 @@
       </c>
       <c r="C27" s="20" t="n"/>
       <c r="D27" s="22" t="n">
-        <v>523.784</v>
+        <v>50000</v>
       </c>
       <c r="E27" s="23" t="n"/>
       <c r="F27" s="23" t="n"/>
@@ -898,7 +882,7 @@
       </c>
       <c r="C28" s="20" t="n"/>
       <c r="D28" s="22" t="n">
-        <v>616.561</v>
+        <v>305.67</v>
       </c>
       <c r="E28" s="23" t="n"/>
       <c r="F28" s="23" t="n"/>
@@ -917,7 +901,7 @@
       </c>
       <c r="C29" s="20" t="n"/>
       <c r="D29" s="22" t="n">
-        <v>1065.765</v>
+        <v>528.38</v>
       </c>
       <c r="E29" s="23" t="n"/>
       <c r="F29" s="23" t="n"/>
@@ -936,7 +920,7 @@
       </c>
       <c r="C30" s="20" t="n"/>
       <c r="D30" s="22" t="n">
-        <v>1314.95</v>
+        <v>651.92</v>
       </c>
       <c r="E30" s="23" t="n"/>
       <c r="F30" s="23" t="n"/>
@@ -955,7 +939,7 @@
       </c>
       <c r="C31" s="20" t="n"/>
       <c r="D31" s="22" t="n">
-        <v>1744.175</v>
+        <v>864.72</v>
       </c>
       <c r="E31" s="23" t="n"/>
       <c r="F31" s="23" t="n"/>
@@ -974,7 +958,7 @@
       </c>
       <c r="C32" s="20" t="n"/>
       <c r="D32" s="22" t="n">
-        <v>2480.758</v>
+        <v>1229.9</v>
       </c>
       <c r="E32" s="23" t="n"/>
       <c r="F32" s="23" t="n"/>
@@ -993,7 +977,7 @@
       </c>
       <c r="C33" s="20" t="n"/>
       <c r="D33" s="22" t="n">
-        <v>3673.842</v>
+        <v>1821.4</v>
       </c>
       <c r="E33" s="23" t="n"/>
       <c r="F33" s="23" t="n"/>
@@ -1033,7 +1017,7 @@
       </c>
       <c r="C35" s="20" t="n"/>
       <c r="D35" s="22" t="n">
-        <v>772.954</v>
+        <v>383.21</v>
       </c>
       <c r="E35" s="23" t="n"/>
       <c r="F35" s="23" t="n"/>
@@ -1052,7 +1036,7 @@
       </c>
       <c r="C36" s="20" t="n"/>
       <c r="D36" s="22" t="n">
-        <v>874.814</v>
+        <v>433.71</v>
       </c>
       <c r="E36" s="23" t="n"/>
       <c r="F36" s="23" t="n"/>
@@ -1071,7 +1055,7 @@
       </c>
       <c r="C37" s="20" t="n"/>
       <c r="D37" s="22" t="n">
-        <v>1116.707</v>
+        <v>553.63</v>
       </c>
       <c r="E37" s="23" t="n"/>
       <c r="F37" s="23" t="n"/>
@@ -1090,7 +1074,7 @@
       </c>
       <c r="C38" s="20" t="n"/>
       <c r="D38" s="22" t="n">
-        <v>1855.127</v>
+        <v>919.72</v>
       </c>
       <c r="E38" s="23" t="n"/>
       <c r="F38" s="23" t="n"/>
@@ -1109,7 +1093,7 @@
       </c>
       <c r="C39" s="20" t="n"/>
       <c r="D39" s="22" t="n">
-        <v>2406.178</v>
+        <v>1192.92</v>
       </c>
       <c r="E39" s="23" t="n"/>
       <c r="F39" s="23" t="n"/>
@@ -1128,7 +1112,7 @@
       </c>
       <c r="C40" s="20" t="n"/>
       <c r="D40" s="22" t="n">
-        <v>3068.195</v>
+        <v>1521.13</v>
       </c>
       <c r="E40" s="23" t="n"/>
       <c r="F40" s="23" t="n"/>
@@ -1147,7 +1131,7 @@
       </c>
       <c r="C41" s="20" t="n"/>
       <c r="D41" s="22" t="n">
-        <v>4314.029</v>
+        <v>2138.79</v>
       </c>
       <c r="E41" s="23" t="n"/>
       <c r="F41" s="23" t="n"/>
@@ -1166,7 +1150,7 @@
       </c>
       <c r="C42" s="20" t="n"/>
       <c r="D42" s="22" t="n">
-        <v>6656.547</v>
+        <v>3300.15</v>
       </c>
       <c r="E42" s="23" t="n"/>
       <c r="F42" s="23" t="n"/>
@@ -1189,12 +1173,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
         <is>
@@ -1204,28 +1182,28 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>